<commit_message>
Stabilize TrackScore before React Phase B
</commit_message>
<xml_diff>
--- a/qa/stabilization/export.xlsx
+++ b/qa/stabilization/export.xlsx
@@ -112,475 +112,475 @@
     <t>Package 1: Standard Assessment (RM 4,500)</t>
   </si>
   <si>
-    <t>2026-10-15T01:52:22.267Z</t>
+    <t>2026-10-17T03:10:17.427Z</t>
   </si>
   <si>
     <t>Completed On Time</t>
   </si>
   <si>
+    <t>Completed on time (9 days ahead)</t>
+  </si>
+  <si>
+    <t>STB 0001</t>
+  </si>
+  <si>
+    <t>Stability Assessor</t>
+  </si>
+  <si>
+    <t>3.50</t>
+  </si>
+  <si>
+    <t>1.50</t>
+  </si>
+  <si>
+    <t>5.00</t>
+  </si>
+  <si>
+    <t>5 Stars - Outstanding (MIROS Certified Grade A)</t>
+  </si>
+  <si>
+    <t>2.0</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>completed</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.012Z</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:11:09.337Z</t>
+  </si>
+  <si>
+    <t>pagination-24</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 24</t>
+  </si>
+  <si>
+    <t>Pager 24</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.011Z</t>
+  </si>
+  <si>
+    <t>pagination-23</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 23</t>
+  </si>
+  <si>
+    <t>Pager 23</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.010Z</t>
+  </si>
+  <si>
+    <t>pagination-22</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 22</t>
+  </si>
+  <si>
+    <t>Pager 22</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.009Z</t>
+  </si>
+  <si>
+    <t>pagination-21</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 21</t>
+  </si>
+  <si>
+    <t>Pager 21</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.008Z</t>
+  </si>
+  <si>
+    <t>pagination-20</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 20</t>
+  </si>
+  <si>
+    <t>Pager 20</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.007Z</t>
+  </si>
+  <si>
+    <t>pagination-19</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 19</t>
+  </si>
+  <si>
+    <t>Pager 19</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.006Z</t>
+  </si>
+  <si>
+    <t>pagination-18</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 18</t>
+  </si>
+  <si>
+    <t>Pager 18</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.005Z</t>
+  </si>
+  <si>
+    <t>pagination-17</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 17</t>
+  </si>
+  <si>
+    <t>Pager 17</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.004Z</t>
+  </si>
+  <si>
+    <t>pagination-16</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 16</t>
+  </si>
+  <si>
+    <t>Pager 16</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.003Z</t>
+  </si>
+  <si>
+    <t>pagination-15</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 15</t>
+  </si>
+  <si>
+    <t>Pager 15</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.002Z</t>
+  </si>
+  <si>
+    <t>pagination-14</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 14</t>
+  </si>
+  <si>
+    <t>Pager 14</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.001Z</t>
+  </si>
+  <si>
+    <t>pagination-13</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 13</t>
+  </si>
+  <si>
+    <t>Pager 13</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:22.000Z</t>
+  </si>
+  <si>
+    <t>pagination-12</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 12</t>
+  </si>
+  <si>
+    <t>Pager 12</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.999Z</t>
+  </si>
+  <si>
+    <t>pagination-11</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 11</t>
+  </si>
+  <si>
+    <t>Pager 11</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.998Z</t>
+  </si>
+  <si>
+    <t>pagination-10</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 10</t>
+  </si>
+  <si>
+    <t>Pager 10</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.997Z</t>
+  </si>
+  <si>
+    <t>pagination-9</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 9</t>
+  </si>
+  <si>
+    <t>Pager 9</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.996Z</t>
+  </si>
+  <si>
+    <t>pagination-8</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 8</t>
+  </si>
+  <si>
+    <t>Pager 8</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.995Z</t>
+  </si>
+  <si>
+    <t>pagination-7</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 7</t>
+  </si>
+  <si>
+    <t>Pager 7</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.994Z</t>
+  </si>
+  <si>
+    <t>pagination-6</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 6</t>
+  </si>
+  <si>
+    <t>Pager 6</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.993Z</t>
+  </si>
+  <si>
+    <t>pagination-5</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 5</t>
+  </si>
+  <si>
+    <t>Pager 5</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.992Z</t>
+  </si>
+  <si>
+    <t>pagination-4</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 4</t>
+  </si>
+  <si>
+    <t>Pager 4</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.991Z</t>
+  </si>
+  <si>
+    <t>pagination-3</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 3</t>
+  </si>
+  <si>
+    <t>Pager 3</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.990Z</t>
+  </si>
+  <si>
+    <t>pagination-2</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 2</t>
+  </si>
+  <si>
+    <t>Pager 2</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.989Z</t>
+  </si>
+  <si>
+    <t>pagination-1</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 1</t>
+  </si>
+  <si>
+    <t>Pager 1</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.988Z</t>
+  </si>
+  <si>
+    <t>pagination-0</t>
+  </si>
+  <si>
+    <t>Pagination Fleet 0</t>
+  </si>
+  <si>
+    <t>Pager 0</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:12:21.987Z</t>
+  </si>
+  <si>
+    <t>stab-registered</t>
+  </si>
+  <si>
+    <t>Stability registered Fleet</t>
+  </si>
+  <si>
+    <t>Stability Gateway registered</t>
+  </si>
+  <si>
+    <t>On Track</t>
+  </si>
+  <si>
+    <t>6 days remaining</t>
+  </si>
+  <si>
+    <t>0.00</t>
+  </si>
+  <si>
+    <t>1.0.0</t>
+  </si>
+  <si>
+    <t>registered</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:10:17.427Z</t>
+  </si>
+  <si>
+    <t>stab-scheduled</t>
+  </si>
+  <si>
+    <t>Stability scheduled Fleet</t>
+  </si>
+  <si>
+    <t>Stability Gateway scheduled</t>
+  </si>
+  <si>
+    <t>scheduled</t>
+  </si>
+  <si>
+    <t>stab-assigned</t>
+  </si>
+  <si>
+    <t>Stability assigned Fleet</t>
+  </si>
+  <si>
+    <t>Stability Gateway assigned</t>
+  </si>
+  <si>
+    <t>pending_review</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:11:09.078Z</t>
+  </si>
+  <si>
+    <t>stab-in_progress</t>
+  </si>
+  <si>
+    <t>Stability in_progress Fleet</t>
+  </si>
+  <si>
+    <t>Stability Gateway in_progress</t>
+  </si>
+  <si>
+    <t>in_progress</t>
+  </si>
+  <si>
+    <t>stab-submitted</t>
+  </si>
+  <si>
+    <t>Stability submitted Fleet</t>
+  </si>
+  <si>
+    <t>Stability Gateway submitted</t>
+  </si>
+  <si>
+    <t>submitted</t>
+  </si>
+  <si>
+    <t>stab-pending_review</t>
+  </si>
+  <si>
+    <t>Stability pending_review Fleet</t>
+  </si>
+  <si>
+    <t>Stability Gateway pending_review</t>
+  </si>
+  <si>
+    <t>stab-rejected</t>
+  </si>
+  <si>
+    <t>Stability rejected Fleet</t>
+  </si>
+  <si>
+    <t>Stability Gateway rejected</t>
+  </si>
+  <si>
+    <t>rejected</t>
+  </si>
+  <si>
+    <t>Update criterion evidence</t>
+  </si>
+  <si>
+    <t>stab-approved</t>
+  </si>
+  <si>
+    <t>Stability approved Fleet</t>
+  </si>
+  <si>
+    <t>Stability Gateway approved</t>
+  </si>
+  <si>
+    <t>2026-10-10T03:11:09.237Z</t>
+  </si>
+  <si>
+    <t>stab-preparing</t>
+  </si>
+  <si>
+    <t>Stability preparing Fleet</t>
+  </si>
+  <si>
+    <t>Stability Gateway preparing</t>
+  </si>
+  <si>
     <t>Completed on time (7 days ahead)</t>
-  </si>
-  <si>
-    <t>STB 0001</t>
-  </si>
-  <si>
-    <t>Stability Assessor</t>
-  </si>
-  <si>
-    <t>3.50</t>
-  </si>
-  <si>
-    <t>1.50</t>
-  </si>
-  <si>
-    <t>5.00</t>
-  </si>
-  <si>
-    <t>5 Stars - Outstanding (MIROS Certified Grade A)</t>
-  </si>
-  <si>
-    <t>2.0</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>completed</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.412Z</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:52:23.838Z</t>
-  </si>
-  <si>
-    <t>pagination-24</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 24</t>
-  </si>
-  <si>
-    <t>Pager 24</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.411Z</t>
-  </si>
-  <si>
-    <t>pagination-23</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 23</t>
-  </si>
-  <si>
-    <t>Pager 23</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.410Z</t>
-  </si>
-  <si>
-    <t>pagination-22</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 22</t>
-  </si>
-  <si>
-    <t>Pager 22</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.409Z</t>
-  </si>
-  <si>
-    <t>pagination-21</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 21</t>
-  </si>
-  <si>
-    <t>Pager 21</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.408Z</t>
-  </si>
-  <si>
-    <t>pagination-20</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 20</t>
-  </si>
-  <si>
-    <t>Pager 20</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.407Z</t>
-  </si>
-  <si>
-    <t>pagination-19</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 19</t>
-  </si>
-  <si>
-    <t>Pager 19</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.406Z</t>
-  </si>
-  <si>
-    <t>pagination-18</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 18</t>
-  </si>
-  <si>
-    <t>Pager 18</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.405Z</t>
-  </si>
-  <si>
-    <t>pagination-17</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 17</t>
-  </si>
-  <si>
-    <t>Pager 17</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.404Z</t>
-  </si>
-  <si>
-    <t>pagination-16</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 16</t>
-  </si>
-  <si>
-    <t>Pager 16</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.403Z</t>
-  </si>
-  <si>
-    <t>pagination-15</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 15</t>
-  </si>
-  <si>
-    <t>Pager 15</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.402Z</t>
-  </si>
-  <si>
-    <t>pagination-14</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 14</t>
-  </si>
-  <si>
-    <t>Pager 14</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.401Z</t>
-  </si>
-  <si>
-    <t>pagination-13</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 13</t>
-  </si>
-  <si>
-    <t>Pager 13</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.400Z</t>
-  </si>
-  <si>
-    <t>pagination-12</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 12</t>
-  </si>
-  <si>
-    <t>Pager 12</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.399Z</t>
-  </si>
-  <si>
-    <t>pagination-11</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 11</t>
-  </si>
-  <si>
-    <t>Pager 11</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.398Z</t>
-  </si>
-  <si>
-    <t>pagination-10</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 10</t>
-  </si>
-  <si>
-    <t>Pager 10</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.397Z</t>
-  </si>
-  <si>
-    <t>pagination-9</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 9</t>
-  </si>
-  <si>
-    <t>Pager 9</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.396Z</t>
-  </si>
-  <si>
-    <t>pagination-8</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 8</t>
-  </si>
-  <si>
-    <t>Pager 8</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.395Z</t>
-  </si>
-  <si>
-    <t>pagination-7</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 7</t>
-  </si>
-  <si>
-    <t>Pager 7</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.394Z</t>
-  </si>
-  <si>
-    <t>pagination-6</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 6</t>
-  </si>
-  <si>
-    <t>Pager 6</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.393Z</t>
-  </si>
-  <si>
-    <t>pagination-5</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 5</t>
-  </si>
-  <si>
-    <t>Pager 5</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.392Z</t>
-  </si>
-  <si>
-    <t>pagination-4</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 4</t>
-  </si>
-  <si>
-    <t>Pager 4</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.391Z</t>
-  </si>
-  <si>
-    <t>pagination-3</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 3</t>
-  </si>
-  <si>
-    <t>Pager 3</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.390Z</t>
-  </si>
-  <si>
-    <t>pagination-2</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 2</t>
-  </si>
-  <si>
-    <t>Pager 2</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.389Z</t>
-  </si>
-  <si>
-    <t>pagination-1</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 1</t>
-  </si>
-  <si>
-    <t>Pager 1</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.388Z</t>
-  </si>
-  <si>
-    <t>pagination-0</t>
-  </si>
-  <si>
-    <t>Pagination Fleet 0</t>
-  </si>
-  <si>
-    <t>Pager 0</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:53:35.387Z</t>
-  </si>
-  <si>
-    <t>stab-registered</t>
-  </si>
-  <si>
-    <t>Stability registered Fleet</t>
-  </si>
-  <si>
-    <t>Stability Gateway registered</t>
-  </si>
-  <si>
-    <t>2026-10-15T01:52:22.266Z</t>
-  </si>
-  <si>
-    <t>On Track</t>
-  </si>
-  <si>
-    <t>6 days remaining</t>
-  </si>
-  <si>
-    <t>0.00</t>
-  </si>
-  <si>
-    <t>1.0.0</t>
-  </si>
-  <si>
-    <t>registered</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:52:22.266Z</t>
-  </si>
-  <si>
-    <t>stab-scheduled</t>
-  </si>
-  <si>
-    <t>Stability scheduled Fleet</t>
-  </si>
-  <si>
-    <t>Stability Gateway scheduled</t>
-  </si>
-  <si>
-    <t>scheduled</t>
-  </si>
-  <si>
-    <t>stab-assigned</t>
-  </si>
-  <si>
-    <t>Stability assigned Fleet</t>
-  </si>
-  <si>
-    <t>Stability Gateway assigned</t>
-  </si>
-  <si>
-    <t>pending_review</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:52:23.555Z</t>
-  </si>
-  <si>
-    <t>stab-in_progress</t>
-  </si>
-  <si>
-    <t>Stability in_progress Fleet</t>
-  </si>
-  <si>
-    <t>Stability Gateway in_progress</t>
-  </si>
-  <si>
-    <t>in_progress</t>
-  </si>
-  <si>
-    <t>stab-submitted</t>
-  </si>
-  <si>
-    <t>Stability submitted Fleet</t>
-  </si>
-  <si>
-    <t>Stability Gateway submitted</t>
-  </si>
-  <si>
-    <t>submitted</t>
-  </si>
-  <si>
-    <t>stab-pending_review</t>
-  </si>
-  <si>
-    <t>Stability pending_review Fleet</t>
-  </si>
-  <si>
-    <t>Stability Gateway pending_review</t>
-  </si>
-  <si>
-    <t>stab-rejected</t>
-  </si>
-  <si>
-    <t>Stability rejected Fleet</t>
-  </si>
-  <si>
-    <t>Stability Gateway rejected</t>
-  </si>
-  <si>
-    <t>rejected</t>
-  </si>
-  <si>
-    <t>Update criterion evidence</t>
-  </si>
-  <si>
-    <t>stab-approved</t>
-  </si>
-  <si>
-    <t>Stability approved Fleet</t>
-  </si>
-  <si>
-    <t>Stability Gateway approved</t>
-  </si>
-  <si>
-    <t>2026-10-08T01:52:23.751Z</t>
-  </si>
-  <si>
-    <t>stab-preparing</t>
-  </si>
-  <si>
-    <t>Stability preparing Fleet</t>
-  </si>
-  <si>
-    <t>Stability Gateway preparing</t>
   </si>
   <si>
     <t>approved</t>
@@ -3374,13 +3374,13 @@
         <v>7</v>
       </c>
       <c r="G28" t="s">
+        <v>33</v>
+      </c>
+      <c r="H28" t="s">
         <v>151</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>152</v>
-      </c>
-      <c r="I28" t="s">
-        <v>153</v>
       </c>
       <c r="J28" t="s">
         <v>36</v>
@@ -3389,16 +3389,16 @@
         <v>37</v>
       </c>
       <c r="L28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="M28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="O28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P28">
         <v>1</v>
@@ -3407,13 +3407,13 @@
         <v>45</v>
       </c>
       <c r="R28" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="S28" t="s">
         <v>43</v>
       </c>
       <c r="T28" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="U28" t="s">
         <v>45</v>
@@ -3434,7 +3434,7 @@
         <v>0</v>
       </c>
       <c r="AA28" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB28" t="s">
         <v>45</v>
@@ -3442,16 +3442,16 @@
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B29" t="s">
         <v>29</v>
       </c>
       <c r="C29" t="s">
+        <v>158</v>
+      </c>
+      <c r="D29" t="s">
         <v>159</v>
-      </c>
-      <c r="D29" t="s">
-        <v>160</v>
       </c>
       <c r="E29" t="s">
         <v>32</v>
@@ -3460,13 +3460,13 @@
         <v>7</v>
       </c>
       <c r="G29" t="s">
+        <v>33</v>
+      </c>
+      <c r="H29" t="s">
         <v>151</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>152</v>
-      </c>
-      <c r="I29" t="s">
-        <v>153</v>
       </c>
       <c r="J29" t="s">
         <v>36</v>
@@ -3475,16 +3475,16 @@
         <v>37</v>
       </c>
       <c r="L29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="M29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="O29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P29">
         <v>1</v>
@@ -3493,13 +3493,13 @@
         <v>45</v>
       </c>
       <c r="R29" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="S29" t="s">
         <v>43</v>
       </c>
       <c r="T29" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="U29" t="s">
         <v>45</v>
@@ -3520,7 +3520,7 @@
         <v>0</v>
       </c>
       <c r="AA29" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB29" t="s">
         <v>45</v>
@@ -3528,16 +3528,16 @@
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B30" t="s">
         <v>29</v>
       </c>
       <c r="C30" t="s">
+        <v>162</v>
+      </c>
+      <c r="D30" t="s">
         <v>163</v>
-      </c>
-      <c r="D30" t="s">
-        <v>164</v>
       </c>
       <c r="E30" t="s">
         <v>32</v>
@@ -3549,10 +3549,10 @@
         <v>33</v>
       </c>
       <c r="H30" t="s">
+        <v>151</v>
+      </c>
+      <c r="I30" t="s">
         <v>152</v>
-      </c>
-      <c r="I30" t="s">
-        <v>153</v>
       </c>
       <c r="J30" t="s">
         <v>36</v>
@@ -3585,7 +3585,7 @@
         <v>43</v>
       </c>
       <c r="T30" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U30" t="s">
         <v>45</v>
@@ -3606,24 +3606,24 @@
         <v>0</v>
       </c>
       <c r="AA30" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB30" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B31" t="s">
         <v>29</v>
       </c>
       <c r="C31" t="s">
+        <v>167</v>
+      </c>
+      <c r="D31" t="s">
         <v>168</v>
-      </c>
-      <c r="D31" t="s">
-        <v>169</v>
       </c>
       <c r="E31" t="s">
         <v>32</v>
@@ -3635,10 +3635,10 @@
         <v>33</v>
       </c>
       <c r="H31" t="s">
+        <v>151</v>
+      </c>
+      <c r="I31" t="s">
         <v>152</v>
-      </c>
-      <c r="I31" t="s">
-        <v>153</v>
       </c>
       <c r="J31" t="s">
         <v>36</v>
@@ -3647,16 +3647,16 @@
         <v>37</v>
       </c>
       <c r="L31" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="M31" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N31" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="O31" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P31">
         <v>1</v>
@@ -3665,13 +3665,13 @@
         <v>45</v>
       </c>
       <c r="R31" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="S31" t="s">
         <v>43</v>
       </c>
       <c r="T31" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="U31" t="s">
         <v>45</v>
@@ -3692,7 +3692,7 @@
         <v>0</v>
       </c>
       <c r="AA31" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB31" t="s">
         <v>45</v>
@@ -3700,16 +3700,16 @@
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B32" t="s">
         <v>29</v>
       </c>
       <c r="C32" t="s">
+        <v>171</v>
+      </c>
+      <c r="D32" t="s">
         <v>172</v>
-      </c>
-      <c r="D32" t="s">
-        <v>173</v>
       </c>
       <c r="E32" t="s">
         <v>32</v>
@@ -3721,10 +3721,10 @@
         <v>33</v>
       </c>
       <c r="H32" t="s">
+        <v>151</v>
+      </c>
+      <c r="I32" t="s">
         <v>152</v>
-      </c>
-      <c r="I32" t="s">
-        <v>153</v>
       </c>
       <c r="J32" t="s">
         <v>36</v>
@@ -3757,7 +3757,7 @@
         <v>43</v>
       </c>
       <c r="T32" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="U32" t="s">
         <v>45</v>
@@ -3778,7 +3778,7 @@
         <v>0</v>
       </c>
       <c r="AA32" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB32" t="s">
         <v>45</v>
@@ -3786,16 +3786,16 @@
     </row>
     <row r="33" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B33" t="s">
         <v>29</v>
       </c>
       <c r="C33" t="s">
+        <v>175</v>
+      </c>
+      <c r="D33" t="s">
         <v>176</v>
-      </c>
-      <c r="D33" t="s">
-        <v>177</v>
       </c>
       <c r="E33" t="s">
         <v>32</v>
@@ -3807,10 +3807,10 @@
         <v>33</v>
       </c>
       <c r="H33" t="s">
+        <v>151</v>
+      </c>
+      <c r="I33" t="s">
         <v>152</v>
-      </c>
-      <c r="I33" t="s">
-        <v>153</v>
       </c>
       <c r="J33" t="s">
         <v>36</v>
@@ -3843,7 +3843,7 @@
         <v>43</v>
       </c>
       <c r="T33" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U33" t="s">
         <v>45</v>
@@ -3864,7 +3864,7 @@
         <v>0</v>
       </c>
       <c r="AA33" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB33" t="s">
         <v>45</v>
@@ -3872,16 +3872,16 @@
     </row>
     <row r="34" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B34" t="s">
         <v>29</v>
       </c>
       <c r="C34" t="s">
+        <v>178</v>
+      </c>
+      <c r="D34" t="s">
         <v>179</v>
-      </c>
-      <c r="D34" t="s">
-        <v>180</v>
       </c>
       <c r="E34" t="s">
         <v>32</v>
@@ -3893,10 +3893,10 @@
         <v>33</v>
       </c>
       <c r="H34" t="s">
+        <v>151</v>
+      </c>
+      <c r="I34" t="s">
         <v>152</v>
-      </c>
-      <c r="I34" t="s">
-        <v>153</v>
       </c>
       <c r="J34" t="s">
         <v>36</v>
@@ -3929,16 +3929,16 @@
         <v>43</v>
       </c>
       <c r="T34" t="s">
+        <v>180</v>
+      </c>
+      <c r="U34" t="s">
+        <v>45</v>
+      </c>
+      <c r="V34" t="s">
+        <v>45</v>
+      </c>
+      <c r="W34" t="s">
         <v>181</v>
-      </c>
-      <c r="U34" t="s">
-        <v>45</v>
-      </c>
-      <c r="V34" t="s">
-        <v>45</v>
-      </c>
-      <c r="W34" t="s">
-        <v>182</v>
       </c>
       <c r="X34" t="s">
         <v>45</v>
@@ -3950,7 +3950,7 @@
         <v>0</v>
       </c>
       <c r="AA34" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB34" t="s">
         <v>45</v>
@@ -3958,16 +3958,16 @@
     </row>
     <row r="35" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B35" t="s">
         <v>29</v>
       </c>
       <c r="C35" t="s">
+        <v>183</v>
+      </c>
+      <c r="D35" t="s">
         <v>184</v>
-      </c>
-      <c r="D35" t="s">
-        <v>185</v>
       </c>
       <c r="E35" t="s">
         <v>32</v>
@@ -4036,24 +4036,24 @@
         <v>4</v>
       </c>
       <c r="AA35" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB35" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B36" t="s">
         <v>29</v>
       </c>
       <c r="C36" t="s">
+        <v>187</v>
+      </c>
+      <c r="D36" t="s">
         <v>188</v>
-      </c>
-      <c r="D36" t="s">
-        <v>189</v>
       </c>
       <c r="E36" t="s">
         <v>32</v>
@@ -4068,7 +4068,7 @@
         <v>34</v>
       </c>
       <c r="I36" t="s">
-        <v>35</v>
+        <v>189</v>
       </c>
       <c r="J36" t="s">
         <v>36</v>
@@ -4122,7 +4122,7 @@
         <v>0</v>
       </c>
       <c r="AA36" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB36" t="s">
         <v>45</v>
@@ -4151,10 +4151,10 @@
         <v>33</v>
       </c>
       <c r="H37" t="s">
+        <v>151</v>
+      </c>
+      <c r="I37" t="s">
         <v>152</v>
-      </c>
-      <c r="I37" t="s">
-        <v>153</v>
       </c>
       <c r="J37" t="s">
         <v>36</v>
@@ -4208,7 +4208,7 @@
         <v>0</v>
       </c>
       <c r="AA37" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB37" t="s">
         <v>45</v>
@@ -4294,7 +4294,7 @@
         <v>0</v>
       </c>
       <c r="AA38" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB38" t="s">
         <v>47</v>
@@ -4311,7 +4311,7 @@
         <v>199</v>
       </c>
       <c r="D39" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E39" t="s">
         <v>32</v>
@@ -4323,10 +4323,10 @@
         <v>33</v>
       </c>
       <c r="H39" t="s">
+        <v>151</v>
+      </c>
+      <c r="I39" t="s">
         <v>152</v>
-      </c>
-      <c r="I39" t="s">
-        <v>153</v>
       </c>
       <c r="J39" t="s">
         <v>200</v>
@@ -4359,7 +4359,7 @@
         <v>43</v>
       </c>
       <c r="T39" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="U39" t="s">
         <v>45</v>
@@ -4380,7 +4380,7 @@
         <v>0</v>
       </c>
       <c r="AA39" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB39" t="s">
         <v>45</v>
@@ -4397,7 +4397,7 @@
         <v>203</v>
       </c>
       <c r="D40" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E40" t="s">
         <v>32</v>
@@ -4406,13 +4406,13 @@
         <v>7</v>
       </c>
       <c r="G40" t="s">
+        <v>33</v>
+      </c>
+      <c r="H40" t="s">
         <v>151</v>
       </c>
-      <c r="H40" t="s">
+      <c r="I40" t="s">
         <v>152</v>
-      </c>
-      <c r="I40" t="s">
-        <v>153</v>
       </c>
       <c r="J40" t="s">
         <v>36</v>
@@ -4421,16 +4421,16 @@
         <v>37</v>
       </c>
       <c r="L40" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="M40" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N40" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="O40" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="P40">
         <v>1</v>
@@ -4439,7 +4439,7 @@
         <v>45</v>
       </c>
       <c r="R40" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="S40" t="s">
         <v>43</v>
@@ -4466,7 +4466,7 @@
         <v>0</v>
       </c>
       <c r="AA40" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AB40" t="s">
         <v>45</v>

</xml_diff>